<commit_message>
fix(data): 恢复 equipments.xlsx 的 G 列每级效果（被 stash 操作误覆盖）
xlsx G 列从 git fsck 找回的悬空 stash commit 恢复；重导 json 确认 per_level 一致

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/excel/equipments.xlsx
+++ b/config/excel/equipments.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20371"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F3F8031-7B79-486B-AD40-A174827174B6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02F009D4-69F9-47D7-8680-FB41549F7403}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="79">
   <si>
     <t>名称</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -59,10 +59,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ui展示描述</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>每个子弹1%概率秒杀血量低于30%的小怪</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -195,26 +191,14 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>暴击率+5%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>头盔</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>气力上限+5%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>暴风大剑</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>暴击伤害+10%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>攻击力+20</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -223,26 +207,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>暴击率基础值+5%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>气力上限基础值+5%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>暴击伤害倍率基础值+10%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>移速基础值+10</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>气力回复速度基础值+5%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>丛林甲</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -307,6 +271,70 @@
   </si>
   <si>
     <t>生命+0.5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>攻击力+1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>受击无敌时间+0.05</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>升级每级实际效果</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>受击无敌时间+0.01</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>暴击率+0.05</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>气力上限+10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>移动速度+10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>气力回复速度+3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>划线气力消耗-0.01</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>暴击率+0.01</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>气力上限+2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>攻击力+1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>移动速度+2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>气力回复速度+0.8</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>划线气力消耗-0.002</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>暴击伤害倍率基础值+0.3</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -644,10 +672,9 @@
     <col min="4" max="4" width="8.88671875" style="1" customWidth="1"/>
     <col min="5" max="5" width="8.88671875" style="1"/>
     <col min="6" max="6" width="31.33203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="19.21875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" customWidth="1"/>
-    <col min="10" max="10" width="22.33203125" customWidth="1"/>
-    <col min="11" max="11" width="21.6640625" customWidth="1"/>
+    <col min="7" max="7" width="20.33203125" customWidth="1"/>
+    <col min="8" max="8" width="22.33203125" customWidth="1"/>
+    <col min="9" max="9" width="21.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -655,7 +682,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>4</v>
@@ -670,743 +697,743 @@
         <v>8</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>9</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="B2" s="1">
         <v>0</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="F2" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>38</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="B3" s="1">
         <v>0</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>39</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="B4" s="1">
         <v>0</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>39</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="B5" s="1">
         <v>0</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>39</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="B6" s="1">
         <v>0</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="G6" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="B7" s="1">
         <v>0</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="B8" s="1">
         <v>0</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="B9" s="1">
         <v>0</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B10" s="1">
         <v>0</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B11" s="1">
         <v>0</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B12" s="1">
         <v>0</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="B13" s="1">
         <v>0</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="B14" s="1">
         <v>0</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="B15" s="1">
         <v>0</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="B16" s="1">
         <v>0</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="B17" s="1">
         <v>0</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B18" s="1">
         <v>0</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="F18" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>39</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B19" s="1">
         <v>0</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>52</v>
+        <v>78</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B20" s="1">
         <v>0</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B21" s="1">
         <v>0</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>3</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>3</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B22" s="1">
         <v>0</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B23" s="1">
         <v>0</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B24" s="1">
         <v>0</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B25" s="1">
         <v>0</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="B26" s="1">
         <v>0</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="B27" s="1">
         <v>0</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="B28" s="1">
         <v>0</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="B29" s="1">
         <v>0</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>32</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="B30" s="1">
         <v>0</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>71</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="B31" s="1">
         <v>0</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="B32" s="1">
         <v>0</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="B33" s="1">
         <v>0</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>29</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1427,15 +1454,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1443,23 +1470,23 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1467,7 +1494,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1475,7 +1502,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1483,63 +1510,63 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>